<commit_message>
ajuste função impressão AC para placa de orificio PRIO
</commit_message>
<xml_diff>
--- a/TemplateAC_PO_PRIO.xlsx
+++ b/TemplateAC_PO_PRIO.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kloeco-my.sharepoint.com/personal/thiago_gallinucci_kloeckner_com/Documents/Desktop/Projetos/PRIO - BRAVO/Documentos/PRIO Priority/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsmetering-my.sharepoint.com/personal/m_bandeira_odsenergysolutions_com/Documents/Documents/AC's_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="292" documentId="8_{E556DCB1-4AC1-4D48-92F4-04B860C81537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A171AE4A-55B6-4FF2-8940-D3ED66722472}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{48B00715-AE6F-4799-A44A-9F329ECB32D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3910B216-0CE7-4A52-A71D-85605A760A3C}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="1" xr2:uid="{E90285C4-3768-491F-AE0E-BAEC12B2D818}"/>
+    <workbookView xWindow="-14625" yWindow="-16440" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{E90285C4-3768-491F-AE0E-BAEC12B2D818}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Template Formulário" sheetId="10" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Template Formulário'!$A$1:$J$8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Template Formulário'!$B$1:$I$51</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="181">
   <si>
     <t xml:space="preserve">071-TG-1041 Gas to cooler temperature gauge </t>
   </si>
@@ -489,23 +489,12 @@
     <t>1.1 Descrição dos itens a serem verificados</t>
   </si>
   <si>
-    <t xml:space="preserve">(      )  Sim       (      ) Não
-OBSERVAÇÕES: </t>
-  </si>
-  <si>
-    <t>(      )  Sim       (      ) Não*
-*Caso a resposta seja “Não”, justifique:</t>
-  </si>
-  <si>
     <t>Responsável pela análise</t>
   </si>
   <si>
     <t>Data:</t>
   </si>
   <si>
-    <t>/</t>
-  </si>
-  <si>
     <t>Número de série:</t>
   </si>
   <si>
@@ -546,9 +535,6 @@
   </si>
   <si>
     <t>v) Medida de planeza/planicidade.</t>
-  </si>
-  <si>
-    <t>w) Medida de ângulo do chanfro “φ”.</t>
   </si>
   <si>
     <t>x) O certificado informa da aprovação/reprovação da placa conforme a norma de referência?</t>
@@ -582,7 +568,25 @@
     <t>d) CE/SAP da placa.</t>
   </si>
   <si>
-    <t>Documento Principal: PRIO-00.02-MDF-PRO-0030 - Verificar Metrologicamente Equipamentos de Medição – Sistema de Gestão de Medição (SGM)</t>
+    <t>ODS Metering Systems</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(   x   )  Sim       (      ) Não
+OBSERVAÇÕES: </t>
+  </si>
+  <si>
+    <t>(   x   )  Sim       (      ) Não
+OBSERVAÇÕES: Houve alteração do diâmetro da placa no computador de vazão.</t>
+  </si>
+  <si>
+    <t>(   x   )  Sim       (      ) Não*
+*Caso a resposta seja “Não”, justifique:</t>
+  </si>
+  <si>
+    <t>w) Medida de ângulo do chanfro “α”.</t>
   </si>
 </sst>
 </file>
@@ -794,7 +798,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -818,6 +822,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -830,17 +837,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1172,7 +1179,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>160640</xdr:colOff>
+      <xdr:colOff>163815</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>286357</xdr:rowOff>
     </xdr:to>
@@ -1217,12 +1224,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -4529,89 +4532,89 @@
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="2:10">
-      <c r="B4" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
     </row>
     <row r="5" spans="2:10">
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
     </row>
     <row r="6" spans="2:10">
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="21"/>
       <c r="E7" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="F7" s="19"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="20"/>
+        <v>151</v>
+      </c>
+      <c r="F7" s="22"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="24"/>
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="23"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="21"/>
       <c r="E8" s="7" t="s">
         <v>133</v>
       </c>
       <c r="F8" s="22"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="I8" s="24"/>
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="C9" s="22"/>
-      <c r="D9" s="23"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="21"/>
       <c r="E9" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="23"/>
+      <c r="F9" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="24"/>
     </row>
     <row r="11" spans="2:10" ht="15" customHeight="1"/>
     <row r="12" spans="2:10" ht="12.75" customHeight="1">
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="6" t="s">
         <v>136</v>
       </c>
@@ -4623,301 +4626,349 @@
       </c>
     </row>
     <row r="13" spans="2:10">
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="5"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="5"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="5"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="5"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
     <row r="17" spans="2:9">
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="5"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
     </row>
     <row r="18" spans="2:9">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="5"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
     </row>
     <row r="19" spans="2:9">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="29" t="s">
         <v>144</v>
       </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="5"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
     </row>
     <row r="20" spans="2:9">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="29" t="s">
         <v>147</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="5"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
     </row>
     <row r="21" spans="2:9">
-      <c r="B21" s="28" t="s">
-        <v>155</v>
-      </c>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="5"/>
+      <c r="B21" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
     </row>
     <row r="22" spans="2:9">
-      <c r="B22" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="5"/>
+      <c r="B22" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
     </row>
     <row r="23" spans="2:9">
-      <c r="B23" s="28" t="s">
-        <v>157</v>
-      </c>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="5"/>
+      <c r="B23" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
     </row>
     <row r="24" spans="2:9">
-      <c r="B24" s="28" t="s">
-        <v>158</v>
-      </c>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="5"/>
+      <c r="B24" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
     </row>
     <row r="25" spans="2:9">
-      <c r="B25" s="28" t="s">
-        <v>159</v>
-      </c>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="5"/>
+      <c r="B25" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
     </row>
     <row r="26" spans="2:9">
-      <c r="B26" s="28" t="s">
-        <v>160</v>
-      </c>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="5"/>
+      <c r="B26" s="29" t="s">
+        <v>157</v>
+      </c>
+      <c r="C26" s="30"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
     </row>
     <row r="27" spans="2:9">
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="5"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
     </row>
     <row r="28" spans="2:9">
-      <c r="B28" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="5"/>
+      <c r="B28" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
     </row>
     <row r="29" spans="2:9">
-      <c r="B29" s="28" t="s">
-        <v>163</v>
-      </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="5"/>
+      <c r="B29" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
     </row>
     <row r="30" spans="2:9">
-      <c r="B30" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="5"/>
+      <c r="B30" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
     </row>
     <row r="31" spans="2:9">
-      <c r="B31" s="28" t="s">
-        <v>164</v>
-      </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="5"/>
+      <c r="B31" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="C31" s="30"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
     </row>
     <row r="32" spans="2:9">
-      <c r="B32" s="28" t="s">
-        <v>165</v>
-      </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="5"/>
+      <c r="B32" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="C32" s="30"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
     </row>
     <row r="33" spans="2:9">
-      <c r="B33" s="28" t="s">
-        <v>166</v>
-      </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="5"/>
+      <c r="B33" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="C33" s="30"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="31"/>
+      <c r="G33" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
     </row>
     <row r="34" spans="2:9">
-      <c r="B34" s="28" t="s">
-        <v>167</v>
-      </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="5"/>
+      <c r="B34" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="31"/>
+      <c r="G34" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
     </row>
     <row r="35" spans="2:9">
-      <c r="B35" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
-      <c r="F35" s="30"/>
-      <c r="G35" s="5"/>
+      <c r="B35" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="31"/>
+      <c r="G35" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
     </row>
     <row r="36" spans="2:9">
-      <c r="B36" s="28" t="s">
-        <v>169</v>
-      </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="5"/>
+      <c r="B36" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="C36" s="30"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H36" s="5"/>
       <c r="I36" s="5"/>
     </row>
     <row r="37" spans="2:9" ht="12.75" customHeight="1">
-      <c r="B37" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="27"/>
+      <c r="B37" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
+      <c r="E37" s="27"/>
+      <c r="F37" s="28"/>
       <c r="G37" s="6" t="s">
         <v>136</v>
       </c>
@@ -4929,148 +4980,156 @@
       </c>
     </row>
     <row r="38" spans="2:9">
-      <c r="B38" s="28" t="s">
-        <v>175</v>
-      </c>
-      <c r="C38" s="29"/>
-      <c r="D38" s="29"/>
-      <c r="E38" s="29"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="5"/>
+      <c r="B38" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="31"/>
+      <c r="G38" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H38" s="5"/>
       <c r="I38" s="5"/>
     </row>
     <row r="39" spans="2:9">
-      <c r="B39" s="28" t="s">
+      <c r="B39" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="17" t="s">
         <v>176</v>
       </c>
-      <c r="C39" s="29"/>
-      <c r="D39" s="29"/>
-      <c r="E39" s="29"/>
-      <c r="F39" s="30"/>
-      <c r="G39" s="5"/>
       <c r="H39" s="5"/>
       <c r="I39" s="5"/>
     </row>
     <row r="40" spans="2:9">
-      <c r="B40" s="28" t="s">
-        <v>177</v>
-      </c>
-      <c r="C40" s="29"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="29"/>
-      <c r="F40" s="30"/>
-      <c r="G40" s="5"/>
+      <c r="B40" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="C40" s="30"/>
+      <c r="D40" s="30"/>
+      <c r="E40" s="30"/>
+      <c r="F40" s="31"/>
+      <c r="G40" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
     </row>
     <row r="41" spans="2:9">
-      <c r="B41" s="28" t="s">
-        <v>178</v>
-      </c>
-      <c r="C41" s="29"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="30"/>
-      <c r="G41" s="5"/>
+      <c r="B41" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30"/>
+      <c r="E41" s="30"/>
+      <c r="F41" s="31"/>
+      <c r="G41" s="17" t="s">
+        <v>176</v>
+      </c>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
     </row>
     <row r="42" spans="2:9" ht="27" customHeight="1">
-      <c r="B42" s="34" t="s">
-        <v>170</v>
-      </c>
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="35"/>
-      <c r="H42" s="35"/>
-      <c r="I42" s="35"/>
+      <c r="B42" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="C42" s="36"/>
+      <c r="D42" s="36"/>
+      <c r="E42" s="36"/>
+      <c r="F42" s="36"/>
+      <c r="G42" s="36"/>
+      <c r="H42" s="36"/>
+      <c r="I42" s="36"/>
     </row>
     <row r="43" spans="2:9" ht="66.75" customHeight="1">
-      <c r="B43" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="33"/>
+      <c r="B43" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="C43" s="33"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="33"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="34"/>
     </row>
     <row r="44" spans="2:9" ht="30.75" customHeight="1">
-      <c r="B44" s="34" t="s">
-        <v>171</v>
-      </c>
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="35"/>
-      <c r="H44" s="35"/>
-      <c r="I44" s="35"/>
+      <c r="B44" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="C44" s="36"/>
+      <c r="D44" s="36"/>
+      <c r="E44" s="36"/>
+      <c r="F44" s="36"/>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="36"/>
     </row>
     <row r="45" spans="2:9" ht="77.25" customHeight="1">
-      <c r="B45" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="C45" s="32"/>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
-      <c r="H45" s="32"/>
-      <c r="I45" s="33"/>
+      <c r="B45" s="32" t="s">
+        <v>178</v>
+      </c>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="33"/>
+      <c r="I45" s="34"/>
     </row>
     <row r="46" spans="2:9" ht="27.75" customHeight="1">
-      <c r="B46" s="34" t="s">
-        <v>172</v>
-      </c>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="35"/>
+      <c r="B46" s="35" t="s">
+        <v>168</v>
+      </c>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="36"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="36"/>
+      <c r="I46" s="36"/>
     </row>
     <row r="47" spans="2:9" ht="63.75" customHeight="1">
-      <c r="B47" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="33"/>
+      <c r="B47" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="34"/>
     </row>
     <row r="48" spans="2:9" ht="28.5" customHeight="1">
-      <c r="B48" s="34" t="s">
-        <v>173</v>
-      </c>
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="35"/>
-      <c r="H48" s="35"/>
-      <c r="I48" s="35"/>
+      <c r="B48" s="35" t="s">
+        <v>169</v>
+      </c>
+      <c r="C48" s="36"/>
+      <c r="D48" s="36"/>
+      <c r="E48" s="36"/>
+      <c r="F48" s="36"/>
+      <c r="G48" s="36"/>
+      <c r="H48" s="36"/>
+      <c r="I48" s="36"/>
     </row>
     <row r="49" spans="2:9" ht="64.5" customHeight="1">
-      <c r="B49" s="36" t="s">
-        <v>150</v>
-      </c>
-      <c r="C49" s="37"/>
-      <c r="D49" s="37"/>
-      <c r="E49" s="37"/>
-      <c r="F49" s="37"/>
-      <c r="G49" s="37"/>
-      <c r="H49" s="37"/>
-      <c r="I49" s="38"/>
+      <c r="B49" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="C49" s="38"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="39"/>
     </row>
     <row r="50" spans="2:9" ht="33" customHeight="1">
       <c r="B50" s="8"/>
@@ -5078,23 +5137,19 @@
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
       <c r="F50" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="G50" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="H50" s="15" t="s">
-        <v>153</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
       <c r="I50" s="16"/>
     </row>
     <row r="51" spans="2:9" ht="36" customHeight="1">
       <c r="B51" s="10"/>
       <c r="C51" s="11"/>
-      <c r="D51" s="39" t="s">
-        <v>151</v>
-      </c>
-      <c r="E51" s="39"/>
+      <c r="D51" s="40" t="s">
+        <v>149</v>
+      </c>
+      <c r="E51" s="40"/>
       <c r="F51" s="11"/>
       <c r="G51" s="11"/>
       <c r="H51" s="11"/>
@@ -5150,7 +5205,7 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="F8:I8"/>
   </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.39370078740157483" footer="0.19685039370078741"/>
   <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
@@ -5386,10 +5441,27 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="573aabb5-4ef4-426a-b8e3-ad71d56fc232"/>
     <ds:schemaRef ds:uri="f68bb4d7-7edc-4d8a-9df8-02dc45d792e0"/>
+    <ds:schemaRef ds:uri="7999d08e-6ea6-4132-9c44-828665d897c8"/>
+    <ds:schemaRef ds:uri="a79d198c-1a72-426e-a584-7aeb6e99d7a7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B799A0EB-4462-4E52-910D-6913A1655207}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B799A0EB-4462-4E52-910D-6913A1655207}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a79d198c-1a72-426e-a584-7aeb6e99d7a7"/>
+    <ds:schemaRef ds:uri="7999d08e-6ea6-4132-9c44-828665d897c8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ajuste de planilhas e regra de novo insturmento
</commit_message>
<xml_diff>
--- a/TemplateAC_PO_PRIO.xlsx
+++ b/TemplateAC_PO_PRIO.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsmetering-my.sharepoint.com/personal/m_bandeira_odsenergysolutions_com/Documents/Documents/AC's_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_7428CB6380031D3E72E9C063AAD480469AA90017" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A86AC440-EC4F-4F3C-9AEB-7404456135A2}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_D24D03330012C02E34A0C2C028C638E3AA53E13D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8798D989-242D-4EA0-961C-FBEC97858756}"/>
   <bookViews>
-    <workbookView xWindow="-14625" yWindow="-16440" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="45" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="Template Formulário" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Template Formulário'!$A$1:$G$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Template Formulário'!$A$1:$I$51</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,21 +37,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="187">
+  <si>
+    <t>Análise crítica de calibração de placas de orifício</t>
+  </si>
   <si>
     <t>Unidade:</t>
   </si>
   <si>
+    <t>FPSO FRADE</t>
+  </si>
+  <si>
     <t>Número de série:</t>
   </si>
   <si>
+    <t>ST‐1954‐PO4444‐P01</t>
+  </si>
+  <si>
     <t>Localização:</t>
   </si>
   <si>
     <t>Número do Certificado:</t>
   </si>
   <si>
+    <t>25‐ODS‐37‐DIM‐022</t>
+  </si>
+  <si>
     <t>Data de Calibração:</t>
+  </si>
+  <si>
+    <t>08/03/2025</t>
   </si>
   <si>
     <t>Empresa Certificadora:</t>
@@ -190,6 +205,9 @@
     <t>Data:</t>
   </si>
   <si>
+    <t>17/03/2026</t>
+  </si>
+  <si>
     <t>Responsável pela análise</t>
   </si>
   <si>
@@ -584,9 +602,6 @@
   </si>
   <si>
     <t>084-5195 CAE-2350 closed drain header isolation valve</t>
-  </si>
-  <si>
-    <t>Análise crítica de calibração de placas de orifício</t>
   </si>
 </sst>
 </file>
@@ -645,8 +660,9 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="22"/>
-      <color rgb="FF007C86"/>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF008080"/>
       <name val="Prio"/>
     </font>
   </fonts>
@@ -664,7 +680,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -786,16 +802,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF0099A8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -813,56 +836,56 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF007C86"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -879,15 +902,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>992725</xdr:colOff>
+      <xdr:colOff>874704</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>74011</xdr:rowOff>
+      <xdr:rowOff>106855</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>459418</xdr:colOff>
+      <xdr:colOff>341397</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>368579</xdr:rowOff>
+      <xdr:rowOff>410948</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -908,8 +931,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6622328" y="225097"/>
-          <a:ext cx="1470228" cy="297743"/>
+          <a:off x="6504307" y="257941"/>
+          <a:ext cx="1470228" cy="304093"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -919,185 +942,6 @@
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>26276</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>6569</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>20145</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>60544</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Rectangle 14">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8D48D0E3-CCB7-45F5-BD45-864FC49904D5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="111673" y="604345"/>
-          <a:ext cx="8671472" cy="53975"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="007C86"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" anchor="ctr"/>
-        <a:lstStyle>
-          <a:defPPr>
-            <a:defRPr lang="pt-BR"/>
-          </a:defPPr>
-          <a:lvl1pPr algn="l" rtl="0" fontAlgn="base">
-            <a:spcBef>
-              <a:spcPct val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPct val="0"/>
-            </a:spcAft>
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl1pPr>
-          <a:lvl2pPr marL="457200" algn="l" rtl="0" fontAlgn="base">
-            <a:spcBef>
-              <a:spcPct val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPct val="0"/>
-            </a:spcAft>
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl2pPr>
-          <a:lvl3pPr marL="914400" algn="l" rtl="0" fontAlgn="base">
-            <a:spcBef>
-              <a:spcPct val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPct val="0"/>
-            </a:spcAft>
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl3pPr>
-          <a:lvl4pPr marL="1371600" algn="l" rtl="0" fontAlgn="base">
-            <a:spcBef>
-              <a:spcPct val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPct val="0"/>
-            </a:spcAft>
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl4pPr>
-          <a:lvl5pPr marL="1828800" algn="l" rtl="0" fontAlgn="base">
-            <a:spcBef>
-              <a:spcPct val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPct val="0"/>
-            </a:spcAft>
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl5pPr>
-          <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl6pPr>
-          <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl7pPr>
-          <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl8pPr>
-          <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-            <a:defRPr kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri" pitchFamily="34" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="Arial" charset="0"/>
-            </a:defRPr>
-          </a:lvl9pPr>
-        </a:lstStyle>
-        <a:p>
-          <a:endParaRPr lang="pt-BR">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1401,18 +1245,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E143"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="64.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="64.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B1">
         <f t="shared" ref="B1:B32" si="0">SEARCH(" ",A1)</f>
@@ -1433,7 +1277,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B2">
         <f t="shared" si="0"/>
@@ -1454,7 +1298,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B3">
         <f t="shared" si="0"/>
@@ -1475,7 +1319,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B4">
         <f t="shared" si="0"/>
@@ -1496,7 +1340,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <f t="shared" si="0"/>
@@ -1517,7 +1361,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <f t="shared" si="0"/>
@@ -1538,7 +1382,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B7">
         <f t="shared" si="0"/>
@@ -1559,7 +1403,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B8">
         <f t="shared" si="0"/>
@@ -1580,7 +1424,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B9">
         <f t="shared" si="0"/>
@@ -1601,7 +1445,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B10">
         <f t="shared" si="0"/>
@@ -1622,7 +1466,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B11">
         <f t="shared" si="0"/>
@@ -1661,7 +1505,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B13">
         <f t="shared" si="0"/>
@@ -1682,7 +1526,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B14">
         <f t="shared" si="0"/>
@@ -1703,7 +1547,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B15">
         <f t="shared" si="0"/>
@@ -1724,7 +1568,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B16">
         <f t="shared" si="0"/>
@@ -1745,7 +1589,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="B17">
         <f t="shared" si="0"/>
@@ -1766,7 +1610,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B18">
         <f t="shared" si="0"/>
@@ -1805,7 +1649,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B20">
         <f t="shared" si="0"/>
@@ -1826,7 +1670,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B21">
         <f t="shared" si="0"/>
@@ -1847,7 +1691,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="B22">
         <f t="shared" si="0"/>
@@ -1868,7 +1712,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B23">
         <f t="shared" si="0"/>
@@ -1889,7 +1733,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="B24">
         <f t="shared" si="0"/>
@@ -1910,7 +1754,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B25">
         <f t="shared" si="0"/>
@@ -1931,7 +1775,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="B26">
         <f t="shared" si="0"/>
@@ -1952,7 +1796,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B27">
         <f t="shared" si="0"/>
@@ -1973,7 +1817,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B28">
         <f t="shared" si="0"/>
@@ -1994,7 +1838,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B29">
         <f t="shared" si="0"/>
@@ -2015,7 +1859,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B30">
         <f t="shared" si="0"/>
@@ -2036,7 +1880,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B31">
         <f t="shared" si="0"/>
@@ -2075,7 +1919,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B33">
         <f t="shared" ref="B33:B64" si="4">SEARCH(" ",A33)</f>
@@ -2096,7 +1940,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B34">
         <f t="shared" si="4"/>
@@ -2117,7 +1961,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B35">
         <f t="shared" si="4"/>
@@ -2138,7 +1982,7 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B36">
         <f t="shared" si="4"/>
@@ -2159,7 +2003,7 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B37">
         <f t="shared" si="4"/>
@@ -2180,7 +2024,7 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B38">
         <f t="shared" si="4"/>
@@ -2201,7 +2045,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B39">
         <f t="shared" si="4"/>
@@ -2240,7 +2084,7 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B41">
         <f t="shared" si="4"/>
@@ -2261,7 +2105,7 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B42">
         <f t="shared" si="4"/>
@@ -2282,7 +2126,7 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B43">
         <f t="shared" si="4"/>
@@ -2303,7 +2147,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B44">
         <f t="shared" si="4"/>
@@ -2324,7 +2168,7 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B45">
         <f t="shared" si="4"/>
@@ -2345,7 +2189,7 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B46">
         <f t="shared" si="4"/>
@@ -2366,7 +2210,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B47">
         <f t="shared" si="4"/>
@@ -2387,7 +2231,7 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B48">
         <f t="shared" si="4"/>
@@ -2408,7 +2252,7 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B49">
         <f t="shared" si="4"/>
@@ -2429,7 +2273,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="B50">
         <f t="shared" si="4"/>
@@ -2450,7 +2294,7 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B51">
         <f t="shared" si="4"/>
@@ -2489,7 +2333,7 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B53">
         <f t="shared" si="4"/>
@@ -2510,7 +2354,7 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="B54">
         <f t="shared" si="4"/>
@@ -2531,7 +2375,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B55">
         <f t="shared" si="4"/>
@@ -2552,7 +2396,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B56">
         <f t="shared" si="4"/>
@@ -2573,7 +2417,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B57">
         <f t="shared" si="4"/>
@@ -2594,7 +2438,7 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="B58">
         <f t="shared" si="4"/>
@@ -2669,7 +2513,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B62">
         <f t="shared" si="4"/>
@@ -2690,7 +2534,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B63">
         <f t="shared" si="4"/>
@@ -2729,7 +2573,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B65">
         <f t="shared" ref="B65:B96" si="8">SEARCH(" ",A65)</f>
@@ -2750,7 +2594,7 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B66">
         <f t="shared" si="8"/>
@@ -2771,7 +2615,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B67">
         <f t="shared" si="8"/>
@@ -2792,7 +2636,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="B68">
         <f t="shared" si="8"/>
@@ -2813,7 +2657,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B69">
         <f t="shared" si="8"/>
@@ -2834,7 +2678,7 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B70">
         <f t="shared" si="8"/>
@@ -2855,7 +2699,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B71">
         <f t="shared" si="8"/>
@@ -2876,7 +2720,7 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B72">
         <f t="shared" si="8"/>
@@ -2897,7 +2741,7 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B73">
         <f t="shared" si="8"/>
@@ -2918,7 +2762,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B74">
         <f t="shared" si="8"/>
@@ -2939,7 +2783,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B75">
         <f t="shared" si="8"/>
@@ -2960,7 +2804,7 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B76">
         <f t="shared" si="8"/>
@@ -2981,7 +2825,7 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B77">
         <f t="shared" si="8"/>
@@ -3002,7 +2846,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B78">
         <f t="shared" si="8"/>
@@ -3023,7 +2867,7 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B79">
         <f t="shared" si="8"/>
@@ -3044,7 +2888,7 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B80">
         <f t="shared" si="8"/>
@@ -3065,7 +2909,7 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B81">
         <f t="shared" si="8"/>
@@ -3086,7 +2930,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B82">
         <f t="shared" si="8"/>
@@ -3107,7 +2951,7 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B83">
         <f t="shared" si="8"/>
@@ -3128,7 +2972,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B84">
         <f t="shared" si="8"/>
@@ -3149,7 +2993,7 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B85">
         <f t="shared" si="8"/>
@@ -3188,7 +3032,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B87">
         <f t="shared" si="8"/>
@@ -3209,7 +3053,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B88">
         <f t="shared" si="8"/>
@@ -3230,7 +3074,7 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B89">
         <f t="shared" si="8"/>
@@ -3251,7 +3095,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B90">
         <f t="shared" si="8"/>
@@ -3272,7 +3116,7 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B91">
         <f t="shared" si="8"/>
@@ -3293,7 +3137,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B92">
         <f t="shared" si="8"/>
@@ -3314,7 +3158,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B93">
         <f t="shared" si="8"/>
@@ -3335,7 +3179,7 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B94">
         <f t="shared" si="8"/>
@@ -3356,7 +3200,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B95">
         <f t="shared" si="8"/>
@@ -3377,7 +3221,7 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B96">
         <f t="shared" si="8"/>
@@ -3398,7 +3242,7 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B97">
         <f t="shared" ref="B97:B128" si="12">SEARCH(" ",A97)</f>
@@ -3419,7 +3263,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B98">
         <f t="shared" si="12"/>
@@ -3440,7 +3284,7 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B99">
         <f t="shared" si="12"/>
@@ -3461,7 +3305,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B100">
         <f t="shared" si="12"/>
@@ -3482,7 +3326,7 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B101">
         <f t="shared" si="12"/>
@@ -3503,7 +3347,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B102">
         <f t="shared" si="12"/>
@@ -3524,7 +3368,7 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B103">
         <f t="shared" si="12"/>
@@ -3545,7 +3389,7 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B104">
         <f t="shared" si="12"/>
@@ -3566,7 +3410,7 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B105">
         <f t="shared" si="12"/>
@@ -3587,7 +3431,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B106">
         <f t="shared" si="12"/>
@@ -3608,7 +3452,7 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B107">
         <f t="shared" si="12"/>
@@ -3629,7 +3473,7 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B108">
         <f t="shared" si="12"/>
@@ -3668,7 +3512,7 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B110">
         <f t="shared" si="12"/>
@@ -3689,7 +3533,7 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B111">
         <f t="shared" si="12"/>
@@ -3710,7 +3554,7 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B112">
         <f t="shared" si="12"/>
@@ -3731,7 +3575,7 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B113">
         <f t="shared" si="12"/>
@@ -3752,7 +3596,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B114">
         <f t="shared" si="12"/>
@@ -3773,7 +3617,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B115">
         <f t="shared" si="12"/>
@@ -3794,7 +3638,7 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B116">
         <f t="shared" si="12"/>
@@ -3815,7 +3659,7 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B117">
         <f t="shared" si="12"/>
@@ -3836,7 +3680,7 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B118">
         <f t="shared" si="12"/>
@@ -3857,7 +3701,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B119">
         <f t="shared" si="12"/>
@@ -3878,7 +3722,7 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B120">
         <f t="shared" si="12"/>
@@ -3899,7 +3743,7 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B121">
         <f t="shared" si="12"/>
@@ -3920,7 +3764,7 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B122">
         <f t="shared" si="12"/>
@@ -3941,7 +3785,7 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B123">
         <f t="shared" si="12"/>
@@ -3962,7 +3806,7 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B124">
         <f t="shared" si="12"/>
@@ -3983,7 +3827,7 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B125">
         <f t="shared" si="12"/>
@@ -4004,7 +3848,7 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B126">
         <f t="shared" si="12"/>
@@ -4025,7 +3869,7 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B127">
         <f t="shared" si="12"/>
@@ -4046,7 +3890,7 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B128">
         <f t="shared" si="12"/>
@@ -4067,14 +3911,14 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B129">
-        <f t="shared" ref="B129:B143" si="16">SEARCH(" ",A129)</f>
+        <f t="shared" ref="B129:B160" si="16">SEARCH(" ",A129)</f>
         <v>13</v>
       </c>
       <c r="C129" t="str">
-        <f t="shared" ref="C129:C143" si="17">LEFT(A129,B129-1)</f>
+        <f t="shared" ref="C129:C160" si="17">LEFT(A129,B129-1)</f>
         <v>071-SDV-1036</v>
       </c>
       <c r="D129">
@@ -4082,13 +3926,13 @@
         <v>77</v>
       </c>
       <c r="E129" t="str">
-        <f t="shared" ref="E129:E143" si="19">RIGHT(A129,D129-B129)</f>
+        <f t="shared" ref="E129:E160" si="19">RIGHT(A129,D129-B129)</f>
         <v xml:space="preserve">3rd stage discharge outlet pressurization bypass shutdown valve </v>
       </c>
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B130">
         <f t="shared" si="16"/>
@@ -4127,7 +3971,7 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B132">
         <f t="shared" si="16"/>
@@ -4148,7 +3992,7 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B133">
         <f t="shared" si="16"/>
@@ -4169,7 +4013,7 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B134">
         <f t="shared" si="16"/>
@@ -4190,7 +4034,7 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B135">
         <f t="shared" si="16"/>
@@ -4211,7 +4055,7 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B136">
         <f t="shared" si="16"/>
@@ -4232,7 +4076,7 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B137">
         <f t="shared" si="16"/>
@@ -4253,7 +4097,7 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B138">
         <f t="shared" si="16"/>
@@ -4274,7 +4118,7 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B139">
         <f t="shared" si="16"/>
@@ -4295,7 +4139,7 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B140">
         <f t="shared" si="16"/>
@@ -4316,7 +4160,7 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B141">
         <f t="shared" si="16"/>
@@ -4337,7 +4181,7 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B142">
         <f t="shared" si="16"/>
@@ -4358,7 +4202,7 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B143">
         <f t="shared" si="16"/>
@@ -4384,656 +4228,677 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:J49"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A2:J49"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12"/>
   <cols>
-    <col min="1" max="1" width="1.26953125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="23" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.453125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" style="2" customWidth="1"/>
-    <col min="8" max="9" width="8" style="2" customWidth="1"/>
-    <col min="10" max="10" width="9.1796875" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="9.1796875" style="2"/>
+    <col min="1" max="1" width="1.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="1" customWidth="1"/>
+    <col min="8" max="9" width="8" style="1" customWidth="1"/>
+    <col min="10" max="11" width="9.140625" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="35.25" customHeight="1">
-      <c r="B2" s="32" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10">
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="2:10">
-      <c r="B4" s="16"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="2:10" ht="14.5">
-      <c r="B5" s="7" t="s">
+    <row r="2" spans="1:10" ht="35.25" customHeight="1">
+      <c r="B2" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="7" t="s">
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+    </row>
+    <row r="3" spans="1:10" ht="15" customHeight="1">
+      <c r="A3" s="14"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="16"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="B4" s="33"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" ht="15" customHeight="1">
+      <c r="B5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="22"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="20"/>
-    </row>
-    <row r="6" spans="2:10" ht="14.5">
-      <c r="B6" s="7" t="s">
+      <c r="C5" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="28"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="7" t="s">
+      <c r="D5" s="18"/>
+      <c r="E5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="20"/>
-    </row>
-    <row r="7" spans="2:10" ht="14.5">
-      <c r="B7" s="7" t="s">
+      <c r="F5" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="7" t="s">
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="18"/>
+    </row>
+    <row r="6" spans="1:10" ht="15" customHeight="1">
+      <c r="B6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="C6" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="18"/>
+      <c r="E6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="20"/>
-    </row>
-    <row r="9" spans="2:10" ht="15" customHeight="1"/>
-    <row r="10" spans="2:10" ht="12.75" customHeight="1">
-      <c r="B10" s="18" t="s">
+      <c r="F6" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="6" t="s">
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="18"/>
+    </row>
+    <row r="7" spans="1:10" ht="15" customHeight="1">
+      <c r="B7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="I10" s="6" t="s">
+      <c r="C7" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="18"/>
+      <c r="E7" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="2:10" ht="14.5">
-      <c r="B11" s="21" t="s">
+      <c r="F7" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="15" t="s">
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="18"/>
+    </row>
+    <row r="9" spans="1:10" ht="15" customHeight="1"/>
+    <row r="10" spans="1:10" ht="12.75" customHeight="1">
+      <c r="B10" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-    </row>
-    <row r="12" spans="2:10" ht="14.5">
-      <c r="B12" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-    </row>
-    <row r="13" spans="2:10" ht="14.5">
-      <c r="B13" s="21" t="s">
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-    </row>
-    <row r="14" spans="2:10" ht="14.5">
-      <c r="B14" s="21" t="s">
+      <c r="I10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-    </row>
-    <row r="15" spans="2:10" ht="14.5">
-      <c r="B15" s="21" t="s">
+    </row>
+    <row r="11" spans="1:10" ht="15" customHeight="1">
+      <c r="B11" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-    </row>
-    <row r="16" spans="2:10" ht="14.5">
-      <c r="B16" s="21" t="s">
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-    </row>
-    <row r="17" spans="2:9" ht="14.5">
-      <c r="B17" s="21" t="s">
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="1:10" ht="15" customHeight="1">
+      <c r="B12" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-    </row>
-    <row r="18" spans="2:9" ht="14.5">
-      <c r="B18" s="21" t="s">
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:10" ht="15" customHeight="1">
+      <c r="B13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-    </row>
-    <row r="19" spans="2:9" ht="14.5">
-      <c r="B19" s="21" t="s">
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="1:10" ht="15" customHeight="1">
+      <c r="B14" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-    </row>
-    <row r="20" spans="2:9" ht="14.5">
-      <c r="B20" s="21" t="s">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15" spans="1:10" ht="15" customHeight="1">
+      <c r="B15" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-    </row>
-    <row r="21" spans="2:9" ht="14.5">
-      <c r="B21" s="21" t="s">
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16" spans="1:10" ht="15" customHeight="1">
+      <c r="B16" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-    </row>
-    <row r="22" spans="2:9" ht="14.5">
-      <c r="B22" s="21" t="s">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="2:9" ht="15" customHeight="1">
+      <c r="B17" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-    </row>
-    <row r="23" spans="2:9" ht="14.5">
-      <c r="B23" s="21" t="s">
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+    </row>
+    <row r="18" spans="2:9" ht="15" customHeight="1">
+      <c r="B18" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-    </row>
-    <row r="24" spans="2:9" ht="14.5">
-      <c r="B24" s="21" t="s">
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="2:9" ht="15" customHeight="1">
+      <c r="B19" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-    </row>
-    <row r="25" spans="2:9" ht="14.5">
-      <c r="B25" s="21" t="s">
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+    </row>
+    <row r="20" spans="2:9" ht="15" customHeight="1">
+      <c r="B20" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-    </row>
-    <row r="26" spans="2:9" ht="14.5">
-      <c r="B26" s="21" t="s">
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="2:9" ht="15" customHeight="1">
+      <c r="B21" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-    </row>
-    <row r="27" spans="2:9" ht="14.5">
-      <c r="B27" s="21" t="s">
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="2:9" ht="15" customHeight="1">
+      <c r="B22" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-    </row>
-    <row r="28" spans="2:9" ht="14.5">
-      <c r="B28" s="21" t="s">
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+    </row>
+    <row r="23" spans="2:9" ht="15" customHeight="1">
+      <c r="B23" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-    </row>
-    <row r="29" spans="2:9" ht="14.5">
-      <c r="B29" s="21" t="s">
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" spans="2:9" ht="15" customHeight="1">
+      <c r="B24" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-    </row>
-    <row r="30" spans="2:9" ht="14.5">
-      <c r="B30" s="21" t="s">
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+    </row>
+    <row r="25" spans="2:9" ht="15" customHeight="1">
+      <c r="B25" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-    </row>
-    <row r="31" spans="2:9" ht="14.5">
-      <c r="B31" s="21" t="s">
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="2:9" ht="15" customHeight="1">
+      <c r="B26" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-    </row>
-    <row r="32" spans="2:9" ht="14.5">
-      <c r="B32" s="21" t="s">
+      <c r="C26" s="20"/>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="2:9" ht="15" customHeight="1">
+      <c r="B27" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-    </row>
-    <row r="33" spans="2:9" ht="14.5">
-      <c r="B33" s="21" t="s">
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="2:9" ht="15" customHeight="1">
+      <c r="B28" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-    </row>
-    <row r="34" spans="2:9" ht="14.5">
-      <c r="B34" s="21" t="s">
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" spans="2:9" ht="15" customHeight="1">
+      <c r="B29" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+    </row>
+    <row r="30" spans="2:9" ht="15" customHeight="1">
+      <c r="B30" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" s="20"/>
+      <c r="D30" s="20"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+    </row>
+    <row r="31" spans="2:9" ht="15" customHeight="1">
+      <c r="B31" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" s="20"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+    </row>
+    <row r="32" spans="2:9" ht="15" customHeight="1">
+      <c r="B32" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="20"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+    </row>
+    <row r="33" spans="2:9" ht="15" customHeight="1">
+      <c r="B33" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+    </row>
+    <row r="34" spans="2:9" ht="15" customHeight="1">
+      <c r="B34" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" s="20"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
     </row>
     <row r="35" spans="2:9" ht="12.75" customHeight="1">
-      <c r="B35" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="I35" s="6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" ht="14.5">
-      <c r="B36" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-    </row>
-    <row r="37" spans="2:9" ht="14.5">
-      <c r="B37" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-    </row>
-    <row r="38" spans="2:9" ht="14.5">
-      <c r="B38" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
-    </row>
-    <row r="39" spans="2:9" ht="14.5">
-      <c r="B39" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5"/>
+      <c r="B35" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="15" customHeight="1">
+      <c r="B36" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+    </row>
+    <row r="37" spans="2:9" ht="15" customHeight="1">
+      <c r="B37" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+    </row>
+    <row r="38" spans="2:9" ht="15" customHeight="1">
+      <c r="B38" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+    </row>
+    <row r="39" spans="2:9" ht="15" customHeight="1">
+      <c r="B39" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
     </row>
     <row r="40" spans="2:9" ht="27" customHeight="1">
-      <c r="B40" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="19"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="20"/>
+      <c r="B40" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="18"/>
     </row>
     <row r="41" spans="2:9" ht="66.75" customHeight="1">
-      <c r="B41" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="20"/>
+      <c r="B41" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C41" s="20"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="20"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="18"/>
     </row>
     <row r="42" spans="2:9" ht="30.75" customHeight="1">
-      <c r="B42" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="19"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="20"/>
+      <c r="B42" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C42" s="20"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="20"/>
+      <c r="I42" s="18"/>
     </row>
     <row r="43" spans="2:9" ht="77.25" customHeight="1">
-      <c r="B43" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="19"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="20"/>
+      <c r="B43" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43" s="20"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="20"/>
+      <c r="G43" s="20"/>
+      <c r="H43" s="20"/>
+      <c r="I43" s="18"/>
     </row>
     <row r="44" spans="2:9" ht="27.75" customHeight="1">
-      <c r="B44" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="C44" s="19"/>
-      <c r="D44" s="19"/>
-      <c r="E44" s="19"/>
-      <c r="F44" s="19"/>
-      <c r="G44" s="19"/>
-      <c r="H44" s="19"/>
-      <c r="I44" s="20"/>
+      <c r="B44" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C44" s="20"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="20"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="20"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="18"/>
     </row>
     <row r="45" spans="2:9" ht="63.75" customHeight="1">
-      <c r="B45" s="27" t="s">
-        <v>42</v>
-      </c>
-      <c r="C45" s="19"/>
-      <c r="D45" s="19"/>
-      <c r="E45" s="19"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="19"/>
-      <c r="H45" s="19"/>
-      <c r="I45" s="20"/>
+      <c r="B45" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C45" s="20"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="20"/>
+      <c r="F45" s="20"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="20"/>
+      <c r="I45" s="18"/>
     </row>
     <row r="46" spans="2:9" ht="28.5" customHeight="1">
-      <c r="B46" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="20"/>
+      <c r="B46" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="20"/>
+      <c r="G46" s="20"/>
+      <c r="H46" s="20"/>
+      <c r="I46" s="18"/>
     </row>
     <row r="47" spans="2:9" ht="64.5" customHeight="1">
-      <c r="B47" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
-      <c r="I47" s="31"/>
+      <c r="B47" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="23"/>
     </row>
     <row r="48" spans="2:9" ht="33" customHeight="1">
-      <c r="B48" s="8"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G48" s="26"/>
-      <c r="H48" s="19"/>
-      <c r="I48" s="20"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="G48" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H48" s="20"/>
+      <c r="I48" s="18"/>
     </row>
     <row r="49" spans="2:9" ht="36" customHeight="1">
-      <c r="B49" s="10"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="E49" s="19"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="12"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="E49" s="20"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+      <c r="I49" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="47">
-    <mergeCell ref="B47:I47"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F7:I7"/>
+  <mergeCells count="48">
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B4:I4"/>
     <mergeCell ref="D49:E49"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B42:I42"/>
@@ -5049,28 +4914,27 @@
     <mergeCell ref="G48:I48"/>
     <mergeCell ref="B45:I45"/>
     <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B47:I47"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="F7:I7"/>
   </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.39370078740157483" footer="0.19685039370078741"/>
-  <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" scale="77" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ajuste xml PO - metodologia AGA 3
</commit_message>
<xml_diff>
--- a/TemplateAC_PO_PRIO.xlsx
+++ b/TemplateAC_PO_PRIO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odsmetering-my.sharepoint.com/personal/m_bandeira_odsenergysolutions_com/Documents/Documents/AC's_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_D24D033300128FC636860A812FC638E3AA53E1E3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB7FD86D-B16D-4FF9-9149-94B5362EFBCD}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_024E72CFC11EA9B67482E0222004F0E59DD3E1E2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{786CB506-2B43-44F6-9FE7-8597329B9D27}"/>
   <bookViews>
-    <workbookView xWindow="13320" yWindow="-16485" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
@@ -39,19 +39,412 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="187">
   <si>
+    <t xml:space="preserve">071-TG-1041 Gas to cooler temperature gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PDI-1080 Gas differential pressure indicator across cooler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PT-1043 Gas to scrubber pressure transmitter </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TSI-1042 Gas to scrubber temperature safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TIC-1043 Gas to scrubber temperature indicator controller </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-PG-1045 Cooling medium supply pressure gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-PDI-1039 C.M. differential pressure indicator across cooler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PG-1015 Scrubber pressure gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-LG-1007 Scrubber level gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-LSI-1013 Scrubber level safety indicator </t>
+  </si>
+  <si>
+    <t>071-LIC-1014 Scrubber level indicator controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PSI-1047 Compressor suction pressure safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TSI-1045 Compressor discharge temperature safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TG-1044 Compressor discharge temperature gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PSI-1048 Compressor discharge pressure safety indicator </t>
+  </si>
+  <si>
+    <t>071-PIC-1049 Compressor suction pressure indicator controller (with high discharge pressure override from 071-PT-1049)</t>
+  </si>
+  <si>
+    <t>071-FI-1027 Compressor discharge flow indicator</t>
+  </si>
+  <si>
+    <t>071-6544 071-SDV-1051 upstream manual valve</t>
+  </si>
+  <si>
+    <t>071-SDV-1051 Flash gas from separators shutdown valve</t>
+  </si>
+  <si>
+    <t>104-6554 Cooling medium supply valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-6555 104-PSV-1043 upstream valve </t>
+  </si>
+  <si>
+    <t>104-TCV-1049 Cooling medium return control valve</t>
+  </si>
+  <si>
+    <t>104-6563 104-TCV-1049 downstream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-6565 071-PSV-1015 upstream valves </t>
+  </si>
+  <si>
+    <t>080-6568 071-PSV-1015 downstream valve</t>
+  </si>
+  <si>
+    <t>084-6573 MBF-2315 bottom drain outlet valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1071 Condensate outlet from MBF-2315 shutdown valve </t>
+  </si>
+  <si>
+    <t>071-LCV-1016 Condensate outlet from MBF-2315 level control valve</t>
+  </si>
+  <si>
+    <t>071-6582 071-LCV-1016 downstream valve</t>
+  </si>
+  <si>
+    <t>071-PCV-1057 Compressor recycle control valve</t>
+  </si>
+  <si>
+    <t>071-6586 071-PSV-1018 upstream valves</t>
+  </si>
+  <si>
+    <t>080-6589 071-PSV-1018 downstream valve</t>
+  </si>
+  <si>
+    <t>071-BDV-1063 Compressor discharge blowdown valve</t>
+  </si>
+  <si>
+    <t>080-6596 071-BDV-1063 downstream valve</t>
+  </si>
+  <si>
+    <t>071-SDV-1052 Compressor discharge shutdown valve</t>
+  </si>
+  <si>
+    <t>071-6594 071-SDV-1052 downstream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TG-1047 Gas to cooler temperature gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PDI-1081 Gas differential pressure indicator across cooler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PT-1051 Gas to scrubber pressure transmitter </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TSI-1048 Gas to scrubber temperature safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TIC-1049 Gas to scrubber temperature indicator controller </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-PG-1046 Cooling medium supply pressure gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-PDI-1040 C.M. differential pressure indicator across cooler </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PG-1016 Scrubber pressure gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-LG-1008 Scrubber level gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-LSI-1015 Scrubber level safety indicator </t>
+  </si>
+  <si>
+    <t>071-LIC-1016 Scrubber level indicator controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PSI-1055 Compressor suction pressure safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TSI-1051 Compressor discharge temperature safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TG-1050 Compressor discharge temperature gauge </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PSI-1056 Compressor discharge pressure safety indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PIC-1057 Compressor suction pressure indicator controller (with high discharge pressure override from 071-PT-1057) </t>
+  </si>
+  <si>
+    <t>071-FI-1028 Compressor discharge flow indicator</t>
+  </si>
+  <si>
+    <t>071-4949 Main compressor 1st stage inlet manual valve</t>
+  </si>
+  <si>
+    <t>071-SDV-1025 Main compressor 1st stage inlet shutdown valve</t>
+  </si>
+  <si>
+    <t>071-SDV-1026 Main compressor 1st stage inlet pressurization bypass shutdown valve</t>
+  </si>
+  <si>
+    <t>071-PCV-1074 Main compressor 1st stage inlet pressure control valve</t>
+  </si>
+  <si>
+    <t>071-4974 071-PSV-1007 up stream valve</t>
+  </si>
+  <si>
+    <t>080-4977 071-PSV-1007 down stream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1027 1st stage suction scrubber MBF-2375 level shutdown valve </t>
+  </si>
+  <si>
+    <t>071-LCV-1008 1st stage suction scrubber MBF-2375 level control valve</t>
+  </si>
+  <si>
+    <t>071-4972 071-LCV-1008 downstream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">084-4959 1st stage suction scrubber MBF-2375 closed drain valve </t>
+  </si>
+  <si>
+    <t>084-4961 1st stage suction scrubber MBF-2375 closed drain header valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-4986 071-SP-2410 1st stage suction sample upstream device </t>
+  </si>
+  <si>
+    <t>071-4990 071-PSV-1008 up stream valve</t>
+  </si>
+  <si>
+    <t>080-4993 071-PSV-1008 down stream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-FCV-1019 1st stage discharge recycle flow control valve (anti-surge control) </t>
+  </si>
+  <si>
+    <t>071-PCV-1098 1st stage discharge recycle flow control valve (capacity control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-4998 Cooling medium supply to HGB-2355 valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-TCV-1026 Temperature control valve on cooling medium return from 1st stage discharge cooler. </t>
+  </si>
+  <si>
+    <t>104-5010 Cooling medium return header valve</t>
+  </si>
+  <si>
+    <t>104-5004 071-PSV-1028 up stream valve</t>
+  </si>
+  <si>
+    <t>071-5030 071-PSV-1009 up stream valve</t>
+  </si>
+  <si>
+    <t>080-5033 071-PSV-1009 down stream valve</t>
+  </si>
+  <si>
+    <t>071-FCV-1022 2nd stage discharge recycle flow control valve (anti-surge control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PCV-1092 2nd stage discharge recycle flow control valve (capacity control) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1028 2nd stage suction scrubber MBF-2390 level shutdown valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-LCV-1010 2nd stage suction scrubber MBF-2390 level control valve </t>
+  </si>
+  <si>
+    <t>071-5028 071-LCV-1010 downstream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">084-5016 2nd stage suction scrubber MBF-2390 closed drain valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">084-5018 2nd stage suction scrubber MBF-2390 closed drain header valve </t>
+  </si>
+  <si>
+    <t>071-5043 071-PSV-1010 up stream valve</t>
+  </si>
+  <si>
+    <t>071-5046 071-PSV-1010 down stream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5061 Cooling medium supply to HGB-2360 valve </t>
+  </si>
+  <si>
+    <t>071-TCV-1034 Temperature control valve on cooling medium return from 2nd stage discharge cooler</t>
+  </si>
+  <si>
+    <t>104-5073 Cooling medium return header valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-BDV-1031 2nd stage discharge blowdown valve </t>
+  </si>
+  <si>
+    <t>071-5075 071-BDV-1031 downstream valve</t>
+  </si>
+  <si>
+    <t>071-5076/77 071-BDV-1031 by-pass valves</t>
+  </si>
+  <si>
+    <t>104-5067 071-PSV-1029 up stream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1029 2nd stage discharge outlet shutdown valve </t>
+  </si>
+  <si>
+    <t>071-SDV-1030 2nd stage discharge outlet pressurization bypass shutdown valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-5060 2nd stage discharge outlet valve </t>
+  </si>
+  <si>
+    <t>071-5078 Main compressor 3rd stage inlet manual valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1032 Main compressor 3rd stage inlet shutdown valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1033 Main compressor 3rd stage inlet pressurization bypass shutdown valve </t>
+  </si>
+  <si>
+    <t>071-PCV-1087 Main compressor 3rd stage inlet pressure control valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-5103 071-PSV-1011 up stream valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-5106 071-PSV-1011 down stream valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1034 3rd stage suction scrubber MBF-2395 level shutdown valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-LCV-1012 3rd stage suction scrubber MBF-2395 level control valve </t>
+  </si>
+  <si>
+    <t>071-5101 071-LCV-1012 downstream valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">084-5089 3rd stage suction scrubber MBF-2395 closed drain valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">084-5091 3rd stage suction scrubber MBF-2395 closed drain header valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-5115 071-SP-2411 3rd stage suction sample upstream isolation device </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-FCV-1024 3rd stage discharge recycle flow control valve (anti-surge control)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-PCV-1084 3rd stage discharge recycle flow control valve (capacity control) </t>
+  </si>
+  <si>
+    <t>071-5118 071-PSV-1012 up stream isolation valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">080-5121 071-PSV-1012 down stream isolation valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5139 Cooling medium supply to HGB-2365 isolation valve </t>
+  </si>
+  <si>
+    <t>071-TCV-1040 Temperature control valve on cooling medium return from 3rd stage discharge cooler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5151 Cooling medium return header isolation valve </t>
+  </si>
+  <si>
+    <t>071-BDV-1038 3rd stage discharge blowdown valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-5136 071-BDV-1038 downstream isolation valve </t>
+  </si>
+  <si>
+    <t>071-5137/38 071-BDV-1038 by-pass valves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1035 3rd stage discharge outlet shutdown isolation valve  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">071-SDV-1036 3rd stage discharge outlet pressurization bypass shutdown valve </t>
+  </si>
+  <si>
+    <t>071-5134 3rd stage discharge outlet isolation valve</t>
+  </si>
+  <si>
+    <t>104-5145 071-PSV-1030 up stream isolation valve</t>
+  </si>
+  <si>
+    <t>071-5135 Ethanol injection point isolation valves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5155 Cooling medium supply to CM-2341 isolation valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5160 Cooling medium return from CM-2341 isolation valve  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5165 Cooling medium supply to ZZZ-2341 isolation valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5168 Cooling medium return from ZZZ-2341 isolation valve </t>
+  </si>
+  <si>
+    <t>084-5177 CAE-2340/45 closed drain header isolation valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5178 Cooling medium supply to CM-2351 isolation valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5183 Cooling medium return from CM-2351 isolation valve </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5184 Cooling medium supply to ZZZ-2351 isolation valve  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">104-5187 Cooling medium return from ZZZ-1351 isolation valve </t>
+  </si>
+  <si>
+    <t>084-5195 CAE-2350 closed drain header isolation valve</t>
+  </si>
+  <si>
     <t>Análise crítica de calibração de placas de orifício</t>
   </si>
   <si>
     <t>Unidade:</t>
   </si>
   <si>
-    <t>ODS LAB</t>
+    <t>ODS Lab</t>
   </si>
   <si>
     <t>Número de série:</t>
   </si>
   <si>
-    <t>CS-PO-21-06-0038</t>
+    <t>CS-PO-18.09-0050</t>
   </si>
   <si>
     <t>Localização:</t>
@@ -60,13 +453,13 @@
     <t>Número do Certificado:</t>
   </si>
   <si>
-    <t>25-ODS-70-DIM-076</t>
+    <t>25-ODS-70-DIM-070</t>
   </si>
   <si>
     <t>Data de Calibração:</t>
   </si>
   <si>
-    <t>12/11/2025</t>
+    <t>27/11/2025</t>
   </si>
   <si>
     <t>Empresa Certificadora:</t>
@@ -205,403 +598,10 @@
     <t>Data:</t>
   </si>
   <si>
-    <t>19/11/2025</t>
+    <t>01/12/2025</t>
   </si>
   <si>
     <t>Responsável pela análise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TG-1041 Gas to cooler temperature gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PDI-1080 Gas differential pressure indicator across cooler </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PT-1043 Gas to scrubber pressure transmitter </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TSI-1042 Gas to scrubber temperature safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TIC-1043 Gas to scrubber temperature indicator controller </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-PG-1045 Cooling medium supply pressure gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-PDI-1039 C.M. differential pressure indicator across cooler </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PG-1015 Scrubber pressure gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-LG-1007 Scrubber level gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-LSI-1013 Scrubber level safety indicator </t>
-  </si>
-  <si>
-    <t>071-LIC-1014 Scrubber level indicator controller</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PSI-1047 Compressor suction pressure safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TSI-1045 Compressor discharge temperature safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TG-1044 Compressor discharge temperature gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PSI-1048 Compressor discharge pressure safety indicator </t>
-  </si>
-  <si>
-    <t>071-PIC-1049 Compressor suction pressure indicator controller (with high discharge pressure override from 071-PT-1049)</t>
-  </si>
-  <si>
-    <t>071-FI-1027 Compressor discharge flow indicator</t>
-  </si>
-  <si>
-    <t>071-6544 071-SDV-1051 upstream manual valve</t>
-  </si>
-  <si>
-    <t>071-SDV-1051 Flash gas from separators shutdown valve</t>
-  </si>
-  <si>
-    <t>104-6554 Cooling medium supply valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-6555 104-PSV-1043 upstream valve </t>
-  </si>
-  <si>
-    <t>104-TCV-1049 Cooling medium return control valve</t>
-  </si>
-  <si>
-    <t>104-6563 104-TCV-1049 downstream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-6565 071-PSV-1015 upstream valves </t>
-  </si>
-  <si>
-    <t>080-6568 071-PSV-1015 downstream valve</t>
-  </si>
-  <si>
-    <t>084-6573 MBF-2315 bottom drain outlet valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1071 Condensate outlet from MBF-2315 shutdown valve </t>
-  </si>
-  <si>
-    <t>071-LCV-1016 Condensate outlet from MBF-2315 level control valve</t>
-  </si>
-  <si>
-    <t>071-6582 071-LCV-1016 downstream valve</t>
-  </si>
-  <si>
-    <t>071-PCV-1057 Compressor recycle control valve</t>
-  </si>
-  <si>
-    <t>071-6586 071-PSV-1018 upstream valves</t>
-  </si>
-  <si>
-    <t>080-6589 071-PSV-1018 downstream valve</t>
-  </si>
-  <si>
-    <t>071-BDV-1063 Compressor discharge blowdown valve</t>
-  </si>
-  <si>
-    <t>080-6596 071-BDV-1063 downstream valve</t>
-  </si>
-  <si>
-    <t>071-SDV-1052 Compressor discharge shutdown valve</t>
-  </si>
-  <si>
-    <t>071-6594 071-SDV-1052 downstream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TG-1047 Gas to cooler temperature gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PDI-1081 Gas differential pressure indicator across cooler </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PT-1051 Gas to scrubber pressure transmitter </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TSI-1048 Gas to scrubber temperature safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TIC-1049 Gas to scrubber temperature indicator controller </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-PG-1046 Cooling medium supply pressure gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-PDI-1040 C.M. differential pressure indicator across cooler </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PG-1016 Scrubber pressure gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-LG-1008 Scrubber level gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-LSI-1015 Scrubber level safety indicator </t>
-  </si>
-  <si>
-    <t>071-LIC-1016 Scrubber level indicator controller</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PSI-1055 Compressor suction pressure safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TSI-1051 Compressor discharge temperature safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TG-1050 Compressor discharge temperature gauge </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PSI-1056 Compressor discharge pressure safety indicator </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PIC-1057 Compressor suction pressure indicator controller (with high discharge pressure override from 071-PT-1057) </t>
-  </si>
-  <si>
-    <t>071-FI-1028 Compressor discharge flow indicator</t>
-  </si>
-  <si>
-    <t>071-4949 Main compressor 1st stage inlet manual valve</t>
-  </si>
-  <si>
-    <t>071-SDV-1025 Main compressor 1st stage inlet shutdown valve</t>
-  </si>
-  <si>
-    <t>071-SDV-1026 Main compressor 1st stage inlet pressurization bypass shutdown valve</t>
-  </si>
-  <si>
-    <t>071-PCV-1074 Main compressor 1st stage inlet pressure control valve</t>
-  </si>
-  <si>
-    <t>071-4974 071-PSV-1007 up stream valve</t>
-  </si>
-  <si>
-    <t>080-4977 071-PSV-1007 down stream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1027 1st stage suction scrubber MBF-2375 level shutdown valve </t>
-  </si>
-  <si>
-    <t>071-LCV-1008 1st stage suction scrubber MBF-2375 level control valve</t>
-  </si>
-  <si>
-    <t>071-4972 071-LCV-1008 downstream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">084-4959 1st stage suction scrubber MBF-2375 closed drain valve </t>
-  </si>
-  <si>
-    <t>084-4961 1st stage suction scrubber MBF-2375 closed drain header valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-4986 071-SP-2410 1st stage suction sample upstream device </t>
-  </si>
-  <si>
-    <t>071-4990 071-PSV-1008 up stream valve</t>
-  </si>
-  <si>
-    <t>080-4993 071-PSV-1008 down stream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-FCV-1019 1st stage discharge recycle flow control valve (anti-surge control) </t>
-  </si>
-  <si>
-    <t>071-PCV-1098 1st stage discharge recycle flow control valve (capacity control)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-4998 Cooling medium supply to HGB-2355 valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-TCV-1026 Temperature control valve on cooling medium return from 1st stage discharge cooler. </t>
-  </si>
-  <si>
-    <t>104-5010 Cooling medium return header valve</t>
-  </si>
-  <si>
-    <t>104-5004 071-PSV-1028 up stream valve</t>
-  </si>
-  <si>
-    <t>071-5030 071-PSV-1009 up stream valve</t>
-  </si>
-  <si>
-    <t>080-5033 071-PSV-1009 down stream valve</t>
-  </si>
-  <si>
-    <t>071-FCV-1022 2nd stage discharge recycle flow control valve (anti-surge control)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PCV-1092 2nd stage discharge recycle flow control valve (capacity control) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1028 2nd stage suction scrubber MBF-2390 level shutdown valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-LCV-1010 2nd stage suction scrubber MBF-2390 level control valve </t>
-  </si>
-  <si>
-    <t>071-5028 071-LCV-1010 downstream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">084-5016 2nd stage suction scrubber MBF-2390 closed drain valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">084-5018 2nd stage suction scrubber MBF-2390 closed drain header valve </t>
-  </si>
-  <si>
-    <t>071-5043 071-PSV-1010 up stream valve</t>
-  </si>
-  <si>
-    <t>071-5046 071-PSV-1010 down stream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5061 Cooling medium supply to HGB-2360 valve </t>
-  </si>
-  <si>
-    <t>071-TCV-1034 Temperature control valve on cooling medium return from 2nd stage discharge cooler</t>
-  </si>
-  <si>
-    <t>104-5073 Cooling medium return header valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-BDV-1031 2nd stage discharge blowdown valve </t>
-  </si>
-  <si>
-    <t>071-5075 071-BDV-1031 downstream valve</t>
-  </si>
-  <si>
-    <t>071-5076/77 071-BDV-1031 by-pass valves</t>
-  </si>
-  <si>
-    <t>104-5067 071-PSV-1029 up stream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1029 2nd stage discharge outlet shutdown valve </t>
-  </si>
-  <si>
-    <t>071-SDV-1030 2nd stage discharge outlet pressurization bypass shutdown valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-5060 2nd stage discharge outlet valve </t>
-  </si>
-  <si>
-    <t>071-5078 Main compressor 3rd stage inlet manual valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1032 Main compressor 3rd stage inlet shutdown valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1033 Main compressor 3rd stage inlet pressurization bypass shutdown valve </t>
-  </si>
-  <si>
-    <t>071-PCV-1087 Main compressor 3rd stage inlet pressure control valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-5103 071-PSV-1011 up stream valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-5106 071-PSV-1011 down stream valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1034 3rd stage suction scrubber MBF-2395 level shutdown valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-LCV-1012 3rd stage suction scrubber MBF-2395 level control valve </t>
-  </si>
-  <si>
-    <t>071-5101 071-LCV-1012 downstream valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">084-5089 3rd stage suction scrubber MBF-2395 closed drain valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">084-5091 3rd stage suction scrubber MBF-2395 closed drain header valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-5115 071-SP-2411 3rd stage suction sample upstream isolation device </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-FCV-1024 3rd stage discharge recycle flow control valve (anti-surge control)  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-PCV-1084 3rd stage discharge recycle flow control valve (capacity control) </t>
-  </si>
-  <si>
-    <t>071-5118 071-PSV-1012 up stream isolation valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">080-5121 071-PSV-1012 down stream isolation valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5139 Cooling medium supply to HGB-2365 isolation valve </t>
-  </si>
-  <si>
-    <t>071-TCV-1040 Temperature control valve on cooling medium return from 3rd stage discharge cooler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5151 Cooling medium return header isolation valve </t>
-  </si>
-  <si>
-    <t>071-BDV-1038 3rd stage discharge blowdown valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-5136 071-BDV-1038 downstream isolation valve </t>
-  </si>
-  <si>
-    <t>071-5137/38 071-BDV-1038 by-pass valves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1035 3rd stage discharge outlet shutdown isolation valve  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">071-SDV-1036 3rd stage discharge outlet pressurization bypass shutdown valve </t>
-  </si>
-  <si>
-    <t>071-5134 3rd stage discharge outlet isolation valve</t>
-  </si>
-  <si>
-    <t>104-5145 071-PSV-1030 up stream isolation valve</t>
-  </si>
-  <si>
-    <t>071-5135 Ethanol injection point isolation valves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5155 Cooling medium supply to CM-2341 isolation valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5160 Cooling medium return from CM-2341 isolation valve  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5165 Cooling medium supply to ZZZ-2341 isolation valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5168 Cooling medium return from ZZZ-2341 isolation valve </t>
-  </si>
-  <si>
-    <t>084-5177 CAE-2340/45 closed drain header isolation valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5178 Cooling medium supply to CM-2351 isolation valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5183 Cooling medium return from CM-2351 isolation valve </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5184 Cooling medium supply to ZZZ-2351 isolation valve  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">104-5187 Cooling medium return from ZZZ-1351 isolation valve </t>
-  </si>
-  <si>
-    <t>084-5195 CAE-2350 closed drain header isolation valve</t>
   </si>
 </sst>
 </file>
@@ -817,7 +817,6 @@
   </cellStyleXfs>
   <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -839,6 +838,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1245,18 +1245,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E143"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="64.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="3.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="64.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="B1">
         <f t="shared" ref="B1:B32" si="0">SEARCH(" ",A1)</f>
@@ -1277,7 +1277,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <f t="shared" si="0"/>
@@ -1298,7 +1298,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <f t="shared" si="0"/>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <f t="shared" si="0"/>
@@ -1340,7 +1340,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <f t="shared" si="0"/>
@@ -1361,7 +1361,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <f t="shared" si="0"/>
@@ -1382,7 +1382,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <f t="shared" si="0"/>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <f t="shared" si="0"/>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <f t="shared" si="0"/>
@@ -1445,7 +1445,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <f t="shared" si="0"/>
@@ -1466,7 +1466,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <f t="shared" si="0"/>
@@ -1505,7 +1505,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>67</v>
+        <v>11</v>
       </c>
       <c r="B13">
         <f t="shared" si="0"/>
@@ -1526,7 +1526,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="B14">
         <f t="shared" si="0"/>
@@ -1547,7 +1547,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <f t="shared" si="0"/>
@@ -1568,7 +1568,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="B16">
         <f t="shared" si="0"/>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="B17">
         <f t="shared" si="0"/>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="B18">
         <f t="shared" si="0"/>
@@ -1649,7 +1649,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="B20">
         <f t="shared" si="0"/>
@@ -1670,7 +1670,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="B21">
         <f t="shared" si="0"/>
@@ -1691,7 +1691,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="B22">
         <f t="shared" si="0"/>
@@ -1712,7 +1712,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="B23">
         <f t="shared" si="0"/>
@@ -1733,7 +1733,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>21</v>
       </c>
       <c r="B24">
         <f t="shared" si="0"/>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>22</v>
       </c>
       <c r="B25">
         <f t="shared" si="0"/>
@@ -1775,7 +1775,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="B26">
         <f t="shared" si="0"/>
@@ -1796,7 +1796,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="B27">
         <f t="shared" si="0"/>
@@ -1817,7 +1817,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="B28">
         <f t="shared" si="0"/>
@@ -1838,7 +1838,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="B29">
         <f t="shared" si="0"/>
@@ -1859,7 +1859,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="B30">
         <f t="shared" si="0"/>
@@ -1880,7 +1880,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="B31">
         <f t="shared" si="0"/>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="B33">
         <f t="shared" ref="B33:B64" si="4">SEARCH(" ",A33)</f>
@@ -1940,7 +1940,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="B34">
         <f t="shared" si="4"/>
@@ -1961,7 +1961,7 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="B35">
         <f t="shared" si="4"/>
@@ -1982,7 +1982,7 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="B36">
         <f t="shared" si="4"/>
@@ -2003,7 +2003,7 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="B37">
         <f t="shared" si="4"/>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="B38">
         <f t="shared" si="4"/>
@@ -2045,7 +2045,7 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="B39">
         <f t="shared" si="4"/>
@@ -2084,7 +2084,7 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="B41">
         <f t="shared" si="4"/>
@@ -2105,7 +2105,7 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>93</v>
+        <v>37</v>
       </c>
       <c r="B42">
         <f t="shared" si="4"/>
@@ -2126,7 +2126,7 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="B43">
         <f t="shared" si="4"/>
@@ -2147,7 +2147,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="B44">
         <f t="shared" si="4"/>
@@ -2168,7 +2168,7 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="B45">
         <f t="shared" si="4"/>
@@ -2189,7 +2189,7 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>97</v>
+        <v>41</v>
       </c>
       <c r="B46">
         <f t="shared" si="4"/>
@@ -2210,7 +2210,7 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>42</v>
       </c>
       <c r="B47">
         <f t="shared" si="4"/>
@@ -2231,7 +2231,7 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>99</v>
+        <v>43</v>
       </c>
       <c r="B48">
         <f t="shared" si="4"/>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="B49">
         <f t="shared" si="4"/>
@@ -2273,7 +2273,7 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>101</v>
+        <v>45</v>
       </c>
       <c r="B50">
         <f t="shared" si="4"/>
@@ -2294,7 +2294,7 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>102</v>
+        <v>46</v>
       </c>
       <c r="B51">
         <f t="shared" si="4"/>
@@ -2333,7 +2333,7 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>47</v>
       </c>
       <c r="B53">
         <f t="shared" si="4"/>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>48</v>
       </c>
       <c r="B54">
         <f t="shared" si="4"/>
@@ -2375,7 +2375,7 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="B55">
         <f t="shared" si="4"/>
@@ -2396,7 +2396,7 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>50</v>
       </c>
       <c r="B56">
         <f t="shared" si="4"/>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>51</v>
       </c>
       <c r="B57">
         <f t="shared" si="4"/>
@@ -2438,7 +2438,7 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="B58">
         <f t="shared" si="4"/>
@@ -2513,7 +2513,7 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="B62">
         <f t="shared" si="4"/>
@@ -2534,7 +2534,7 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>110</v>
+        <v>54</v>
       </c>
       <c r="B63">
         <f t="shared" si="4"/>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>111</v>
+        <v>55</v>
       </c>
       <c r="B65">
         <f t="shared" ref="B65:B96" si="8">SEARCH(" ",A65)</f>
@@ -2594,7 +2594,7 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="B66">
         <f t="shared" si="8"/>
@@ -2615,7 +2615,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>113</v>
+        <v>57</v>
       </c>
       <c r="B67">
         <f t="shared" si="8"/>
@@ -2636,7 +2636,7 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="B68">
         <f t="shared" si="8"/>
@@ -2657,7 +2657,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>115</v>
+        <v>59</v>
       </c>
       <c r="B69">
         <f t="shared" si="8"/>
@@ -2678,7 +2678,7 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>116</v>
+        <v>60</v>
       </c>
       <c r="B70">
         <f t="shared" si="8"/>
@@ -2699,7 +2699,7 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>117</v>
+        <v>61</v>
       </c>
       <c r="B71">
         <f t="shared" si="8"/>
@@ -2720,7 +2720,7 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="B72">
         <f t="shared" si="8"/>
@@ -2741,7 +2741,7 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>119</v>
+        <v>63</v>
       </c>
       <c r="B73">
         <f t="shared" si="8"/>
@@ -2762,7 +2762,7 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>120</v>
+        <v>64</v>
       </c>
       <c r="B74">
         <f t="shared" si="8"/>
@@ -2783,7 +2783,7 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>121</v>
+        <v>65</v>
       </c>
       <c r="B75">
         <f t="shared" si="8"/>
@@ -2804,7 +2804,7 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>122</v>
+        <v>66</v>
       </c>
       <c r="B76">
         <f t="shared" si="8"/>
@@ -2825,7 +2825,7 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>123</v>
+        <v>67</v>
       </c>
       <c r="B77">
         <f t="shared" si="8"/>
@@ -2846,7 +2846,7 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" t="s">
-        <v>124</v>
+        <v>68</v>
       </c>
       <c r="B78">
         <f t="shared" si="8"/>
@@ -2867,7 +2867,7 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" t="s">
-        <v>125</v>
+        <v>69</v>
       </c>
       <c r="B79">
         <f t="shared" si="8"/>
@@ -2888,7 +2888,7 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" t="s">
-        <v>126</v>
+        <v>70</v>
       </c>
       <c r="B80">
         <f t="shared" si="8"/>
@@ -2909,7 +2909,7 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" t="s">
-        <v>127</v>
+        <v>71</v>
       </c>
       <c r="B81">
         <f t="shared" si="8"/>
@@ -2930,7 +2930,7 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
-        <v>128</v>
+        <v>72</v>
       </c>
       <c r="B82">
         <f t="shared" si="8"/>
@@ -2951,7 +2951,7 @@
     </row>
     <row r="83" spans="1:5">
       <c r="A83" t="s">
-        <v>129</v>
+        <v>73</v>
       </c>
       <c r="B83">
         <f t="shared" si="8"/>
@@ -2972,7 +2972,7 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" t="s">
-        <v>130</v>
+        <v>74</v>
       </c>
       <c r="B84">
         <f t="shared" si="8"/>
@@ -2993,7 +2993,7 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" t="s">
-        <v>131</v>
+        <v>75</v>
       </c>
       <c r="B85">
         <f t="shared" si="8"/>
@@ -3032,7 +3032,7 @@
     </row>
     <row r="87" spans="1:5">
       <c r="A87" t="s">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="B87">
         <f t="shared" si="8"/>
@@ -3053,7 +3053,7 @@
     </row>
     <row r="88" spans="1:5">
       <c r="A88" t="s">
-        <v>133</v>
+        <v>77</v>
       </c>
       <c r="B88">
         <f t="shared" si="8"/>
@@ -3074,7 +3074,7 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>134</v>
+        <v>78</v>
       </c>
       <c r="B89">
         <f t="shared" si="8"/>
@@ -3095,7 +3095,7 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>135</v>
+        <v>79</v>
       </c>
       <c r="B90">
         <f t="shared" si="8"/>
@@ -3116,7 +3116,7 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
       <c r="B91">
         <f t="shared" si="8"/>
@@ -3137,7 +3137,7 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>137</v>
+        <v>81</v>
       </c>
       <c r="B92">
         <f t="shared" si="8"/>
@@ -3158,7 +3158,7 @@
     </row>
     <row r="93" spans="1:5">
       <c r="A93" t="s">
-        <v>138</v>
+        <v>82</v>
       </c>
       <c r="B93">
         <f t="shared" si="8"/>
@@ -3179,7 +3179,7 @@
     </row>
     <row r="94" spans="1:5">
       <c r="A94" t="s">
-        <v>139</v>
+        <v>83</v>
       </c>
       <c r="B94">
         <f t="shared" si="8"/>
@@ -3200,7 +3200,7 @@
     </row>
     <row r="95" spans="1:5">
       <c r="A95" t="s">
-        <v>140</v>
+        <v>84</v>
       </c>
       <c r="B95">
         <f t="shared" si="8"/>
@@ -3221,7 +3221,7 @@
     </row>
     <row r="96" spans="1:5">
       <c r="A96" t="s">
-        <v>141</v>
+        <v>85</v>
       </c>
       <c r="B96">
         <f t="shared" si="8"/>
@@ -3242,7 +3242,7 @@
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>142</v>
+        <v>86</v>
       </c>
       <c r="B97">
         <f t="shared" ref="B97:B128" si="12">SEARCH(" ",A97)</f>
@@ -3263,7 +3263,7 @@
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>143</v>
+        <v>87</v>
       </c>
       <c r="B98">
         <f t="shared" si="12"/>
@@ -3284,7 +3284,7 @@
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>144</v>
+        <v>88</v>
       </c>
       <c r="B99">
         <f t="shared" si="12"/>
@@ -3305,7 +3305,7 @@
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>145</v>
+        <v>89</v>
       </c>
       <c r="B100">
         <f t="shared" si="12"/>
@@ -3326,7 +3326,7 @@
     </row>
     <row r="101" spans="1:5">
       <c r="A101" t="s">
-        <v>146</v>
+        <v>90</v>
       </c>
       <c r="B101">
         <f t="shared" si="12"/>
@@ -3347,7 +3347,7 @@
     </row>
     <row r="102" spans="1:5">
       <c r="A102" t="s">
-        <v>147</v>
+        <v>91</v>
       </c>
       <c r="B102">
         <f t="shared" si="12"/>
@@ -3368,7 +3368,7 @@
     </row>
     <row r="103" spans="1:5">
       <c r="A103" t="s">
-        <v>148</v>
+        <v>92</v>
       </c>
       <c r="B103">
         <f t="shared" si="12"/>
@@ -3389,7 +3389,7 @@
     </row>
     <row r="104" spans="1:5">
       <c r="A104" t="s">
-        <v>149</v>
+        <v>93</v>
       </c>
       <c r="B104">
         <f t="shared" si="12"/>
@@ -3410,7 +3410,7 @@
     </row>
     <row r="105" spans="1:5">
       <c r="A105" t="s">
-        <v>150</v>
+        <v>94</v>
       </c>
       <c r="B105">
         <f t="shared" si="12"/>
@@ -3431,7 +3431,7 @@
     </row>
     <row r="106" spans="1:5">
       <c r="A106" t="s">
-        <v>151</v>
+        <v>95</v>
       </c>
       <c r="B106">
         <f t="shared" si="12"/>
@@ -3452,7 +3452,7 @@
     </row>
     <row r="107" spans="1:5">
       <c r="A107" t="s">
-        <v>152</v>
+        <v>96</v>
       </c>
       <c r="B107">
         <f t="shared" si="12"/>
@@ -3473,7 +3473,7 @@
     </row>
     <row r="108" spans="1:5">
       <c r="A108" t="s">
-        <v>153</v>
+        <v>97</v>
       </c>
       <c r="B108">
         <f t="shared" si="12"/>
@@ -3512,7 +3512,7 @@
     </row>
     <row r="110" spans="1:5">
       <c r="A110" t="s">
-        <v>154</v>
+        <v>98</v>
       </c>
       <c r="B110">
         <f t="shared" si="12"/>
@@ -3533,7 +3533,7 @@
     </row>
     <row r="111" spans="1:5">
       <c r="A111" t="s">
-        <v>155</v>
+        <v>99</v>
       </c>
       <c r="B111">
         <f t="shared" si="12"/>
@@ -3554,7 +3554,7 @@
     </row>
     <row r="112" spans="1:5">
       <c r="A112" t="s">
-        <v>156</v>
+        <v>100</v>
       </c>
       <c r="B112">
         <f t="shared" si="12"/>
@@ -3575,7 +3575,7 @@
     </row>
     <row r="113" spans="1:5">
       <c r="A113" t="s">
-        <v>157</v>
+        <v>101</v>
       </c>
       <c r="B113">
         <f t="shared" si="12"/>
@@ -3596,7 +3596,7 @@
     </row>
     <row r="114" spans="1:5">
       <c r="A114" t="s">
-        <v>158</v>
+        <v>102</v>
       </c>
       <c r="B114">
         <f t="shared" si="12"/>
@@ -3617,7 +3617,7 @@
     </row>
     <row r="115" spans="1:5">
       <c r="A115" t="s">
-        <v>159</v>
+        <v>103</v>
       </c>
       <c r="B115">
         <f t="shared" si="12"/>
@@ -3638,7 +3638,7 @@
     </row>
     <row r="116" spans="1:5">
       <c r="A116" t="s">
-        <v>160</v>
+        <v>104</v>
       </c>
       <c r="B116">
         <f t="shared" si="12"/>
@@ -3659,7 +3659,7 @@
     </row>
     <row r="117" spans="1:5">
       <c r="A117" t="s">
-        <v>161</v>
+        <v>105</v>
       </c>
       <c r="B117">
         <f t="shared" si="12"/>
@@ -3680,7 +3680,7 @@
     </row>
     <row r="118" spans="1:5">
       <c r="A118" t="s">
-        <v>162</v>
+        <v>106</v>
       </c>
       <c r="B118">
         <f t="shared" si="12"/>
@@ -3701,7 +3701,7 @@
     </row>
     <row r="119" spans="1:5">
       <c r="A119" t="s">
-        <v>163</v>
+        <v>107</v>
       </c>
       <c r="B119">
         <f t="shared" si="12"/>
@@ -3722,7 +3722,7 @@
     </row>
     <row r="120" spans="1:5">
       <c r="A120" t="s">
-        <v>164</v>
+        <v>108</v>
       </c>
       <c r="B120">
         <f t="shared" si="12"/>
@@ -3743,7 +3743,7 @@
     </row>
     <row r="121" spans="1:5">
       <c r="A121" t="s">
-        <v>165</v>
+        <v>109</v>
       </c>
       <c r="B121">
         <f t="shared" si="12"/>
@@ -3764,7 +3764,7 @@
     </row>
     <row r="122" spans="1:5">
       <c r="A122" t="s">
-        <v>166</v>
+        <v>110</v>
       </c>
       <c r="B122">
         <f t="shared" si="12"/>
@@ -3785,7 +3785,7 @@
     </row>
     <row r="123" spans="1:5">
       <c r="A123" t="s">
-        <v>167</v>
+        <v>111</v>
       </c>
       <c r="B123">
         <f t="shared" si="12"/>
@@ -3806,7 +3806,7 @@
     </row>
     <row r="124" spans="1:5">
       <c r="A124" t="s">
-        <v>168</v>
+        <v>112</v>
       </c>
       <c r="B124">
         <f t="shared" si="12"/>
@@ -3827,7 +3827,7 @@
     </row>
     <row r="125" spans="1:5">
       <c r="A125" t="s">
-        <v>169</v>
+        <v>113</v>
       </c>
       <c r="B125">
         <f t="shared" si="12"/>
@@ -3848,7 +3848,7 @@
     </row>
     <row r="126" spans="1:5">
       <c r="A126" t="s">
-        <v>170</v>
+        <v>114</v>
       </c>
       <c r="B126">
         <f t="shared" si="12"/>
@@ -3869,7 +3869,7 @@
     </row>
     <row r="127" spans="1:5">
       <c r="A127" t="s">
-        <v>171</v>
+        <v>115</v>
       </c>
       <c r="B127">
         <f t="shared" si="12"/>
@@ -3890,7 +3890,7 @@
     </row>
     <row r="128" spans="1:5">
       <c r="A128" t="s">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="B128">
         <f t="shared" si="12"/>
@@ -3911,7 +3911,7 @@
     </row>
     <row r="129" spans="1:5">
       <c r="A129" t="s">
-        <v>173</v>
+        <v>117</v>
       </c>
       <c r="B129">
         <f t="shared" ref="B129:B160" si="16">SEARCH(" ",A129)</f>
@@ -3932,7 +3932,7 @@
     </row>
     <row r="130" spans="1:5">
       <c r="A130" t="s">
-        <v>174</v>
+        <v>118</v>
       </c>
       <c r="B130">
         <f t="shared" si="16"/>
@@ -3971,7 +3971,7 @@
     </row>
     <row r="132" spans="1:5">
       <c r="A132" t="s">
-        <v>175</v>
+        <v>119</v>
       </c>
       <c r="B132">
         <f t="shared" si="16"/>
@@ -3992,7 +3992,7 @@
     </row>
     <row r="133" spans="1:5">
       <c r="A133" t="s">
-        <v>176</v>
+        <v>120</v>
       </c>
       <c r="B133">
         <f t="shared" si="16"/>
@@ -4013,7 +4013,7 @@
     </row>
     <row r="134" spans="1:5">
       <c r="A134" t="s">
-        <v>177</v>
+        <v>121</v>
       </c>
       <c r="B134">
         <f t="shared" si="16"/>
@@ -4034,7 +4034,7 @@
     </row>
     <row r="135" spans="1:5">
       <c r="A135" t="s">
-        <v>178</v>
+        <v>122</v>
       </c>
       <c r="B135">
         <f t="shared" si="16"/>
@@ -4055,7 +4055,7 @@
     </row>
     <row r="136" spans="1:5">
       <c r="A136" t="s">
-        <v>179</v>
+        <v>123</v>
       </c>
       <c r="B136">
         <f t="shared" si="16"/>
@@ -4076,7 +4076,7 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>180</v>
+        <v>124</v>
       </c>
       <c r="B137">
         <f t="shared" si="16"/>
@@ -4097,7 +4097,7 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
-        <v>181</v>
+        <v>125</v>
       </c>
       <c r="B138">
         <f t="shared" si="16"/>
@@ -4118,7 +4118,7 @@
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>182</v>
+        <v>126</v>
       </c>
       <c r="B139">
         <f t="shared" si="16"/>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="140" spans="1:5">
       <c r="A140" t="s">
-        <v>183</v>
+        <v>127</v>
       </c>
       <c r="B140">
         <f t="shared" si="16"/>
@@ -4160,7 +4160,7 @@
     </row>
     <row r="141" spans="1:5">
       <c r="A141" t="s">
-        <v>184</v>
+        <v>128</v>
       </c>
       <c r="B141">
         <f t="shared" si="16"/>
@@ -4181,7 +4181,7 @@
     </row>
     <row r="142" spans="1:5">
       <c r="A142" t="s">
-        <v>185</v>
+        <v>129</v>
       </c>
       <c r="B142">
         <f t="shared" si="16"/>
@@ -4202,7 +4202,7 @@
     </row>
     <row r="143" spans="1:5">
       <c r="A143" t="s">
-        <v>186</v>
+        <v>130</v>
       </c>
       <c r="B143">
         <f t="shared" si="16"/>
@@ -4232,38 +4232,38 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:J49"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12"/>
   <cols>
-    <col min="1" max="1" width="1.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.453125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.1796875" style="1" customWidth="1"/>
-    <col min="8" max="9" width="8" style="1" customWidth="1"/>
-    <col min="10" max="12" width="9.1796875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.1796875" style="1"/>
+    <col min="1" max="1" width="1.28515625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="23" style="16" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" style="16" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" style="16" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" style="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" style="16" customWidth="1"/>
+    <col min="7" max="7" width="8.140625" style="16" customWidth="1"/>
+    <col min="8" max="9" width="8" style="16" customWidth="1"/>
+    <col min="10" max="14" width="9.140625" style="16" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="16"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="35.25" customHeight="1">
       <c r="B2" s="29" t="s">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
       <c r="E2" s="30"/>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1">
-      <c r="A3" s="14"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="16"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="15"/>
     </row>
     <row r="4" spans="1:10">
       <c r="B4" s="33"/>
@@ -4274,57 +4274,57 @@
       <c r="G4" s="30"/>
       <c r="H4" s="30"/>
       <c r="I4" s="30"/>
-      <c r="J4" s="2"/>
+      <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="B5" s="5" t="s">
-        <v>1</v>
+      <c r="B5" s="4" t="s">
+        <v>132</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>2</v>
+        <v>133</v>
       </c>
       <c r="D5" s="18"/>
-      <c r="E5" s="5" t="s">
-        <v>3</v>
+      <c r="E5" s="4" t="s">
+        <v>134</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>4</v>
+        <v>135</v>
       </c>
       <c r="G5" s="20"/>
       <c r="H5" s="20"/>
       <c r="I5" s="18"/>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1">
-      <c r="B6" s="5" t="s">
-        <v>5</v>
+      <c r="B6" s="4" t="s">
+        <v>136</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>2</v>
+        <v>133</v>
       </c>
       <c r="D6" s="18"/>
-      <c r="E6" s="5" t="s">
-        <v>6</v>
+      <c r="E6" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>7</v>
+        <v>138</v>
       </c>
       <c r="G6" s="20"/>
       <c r="H6" s="20"/>
       <c r="I6" s="18"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
-      <c r="B7" s="5" t="s">
-        <v>8</v>
+      <c r="B7" s="4" t="s">
+        <v>139</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>9</v>
+        <v>140</v>
       </c>
       <c r="D7" s="18"/>
-      <c r="E7" s="5" t="s">
-        <v>10</v>
+      <c r="E7" s="4" t="s">
+        <v>141</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>11</v>
+        <v>142</v>
       </c>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
@@ -4333,435 +4333,435 @@
     <row r="9" spans="1:10" ht="15" customHeight="1"/>
     <row r="10" spans="1:10" ht="12.75" customHeight="1">
       <c r="B10" s="28" t="s">
-        <v>12</v>
+        <v>143</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
       <c r="E10" s="20"/>
       <c r="F10" s="18"/>
-      <c r="G10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>15</v>
+      <c r="G10" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15" customHeight="1">
       <c r="B11" s="19" t="s">
-        <v>16</v>
+        <v>147</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="20"/>
       <c r="E11" s="20"/>
       <c r="F11" s="18"/>
-      <c r="G11" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="G11" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="15" customHeight="1">
       <c r="B12" s="19" t="s">
-        <v>18</v>
+        <v>149</v>
       </c>
       <c r="C12" s="20"/>
       <c r="D12" s="20"/>
       <c r="E12" s="20"/>
       <c r="F12" s="18"/>
-      <c r="G12" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="G12" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1">
       <c r="B13" s="19" t="s">
-        <v>19</v>
+        <v>150</v>
       </c>
       <c r="C13" s="20"/>
       <c r="D13" s="20"/>
       <c r="E13" s="20"/>
       <c r="F13" s="18"/>
-      <c r="G13" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="G13" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1">
       <c r="B14" s="19" t="s">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="C14" s="20"/>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
       <c r="F14" s="18"/>
-      <c r="G14" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="G14" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
       <c r="B15" s="19" t="s">
-        <v>21</v>
+        <v>152</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
       <c r="E15" s="20"/>
       <c r="F15" s="18"/>
-      <c r="G15" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
+      <c r="G15" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="15" customHeight="1">
       <c r="B16" s="19" t="s">
-        <v>22</v>
+        <v>153</v>
       </c>
       <c r="C16" s="20"/>
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
       <c r="F16" s="18"/>
-      <c r="G16" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
+      <c r="G16" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
     </row>
     <row r="17" spans="2:9" ht="15" customHeight="1">
       <c r="B17" s="19" t="s">
-        <v>23</v>
+        <v>154</v>
       </c>
       <c r="C17" s="20"/>
       <c r="D17" s="20"/>
       <c r="E17" s="20"/>
       <c r="F17" s="18"/>
-      <c r="G17" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
+      <c r="G17" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
     </row>
     <row r="18" spans="2:9" ht="15" customHeight="1">
       <c r="B18" s="19" t="s">
-        <v>24</v>
+        <v>155</v>
       </c>
       <c r="C18" s="20"/>
       <c r="D18" s="20"/>
       <c r="E18" s="20"/>
       <c r="F18" s="18"/>
-      <c r="G18" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
+      <c r="G18" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
     </row>
     <row r="19" spans="2:9" ht="15" customHeight="1">
       <c r="B19" s="19" t="s">
-        <v>25</v>
+        <v>156</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="20"/>
       <c r="E19" s="20"/>
       <c r="F19" s="18"/>
-      <c r="G19" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
+      <c r="G19" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
     </row>
     <row r="20" spans="2:9" ht="15" customHeight="1">
       <c r="B20" s="19" t="s">
-        <v>26</v>
+        <v>157</v>
       </c>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
       <c r="E20" s="20"/>
       <c r="F20" s="18"/>
-      <c r="G20" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
+      <c r="G20" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
     </row>
     <row r="21" spans="2:9" ht="15" customHeight="1">
       <c r="B21" s="19" t="s">
-        <v>27</v>
+        <v>158</v>
       </c>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
       <c r="E21" s="20"/>
       <c r="F21" s="18"/>
-      <c r="G21" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
+      <c r="G21" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
     </row>
     <row r="22" spans="2:9" ht="15" customHeight="1">
       <c r="B22" s="19" t="s">
-        <v>28</v>
+        <v>159</v>
       </c>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
       <c r="E22" s="20"/>
       <c r="F22" s="18"/>
-      <c r="G22" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
+      <c r="G22" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
     </row>
     <row r="23" spans="2:9" ht="15" customHeight="1">
       <c r="B23" s="19" t="s">
-        <v>29</v>
+        <v>160</v>
       </c>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
       <c r="E23" s="20"/>
       <c r="F23" s="18"/>
-      <c r="G23" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
+      <c r="G23" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
     </row>
     <row r="24" spans="2:9" ht="15" customHeight="1">
       <c r="B24" s="19" t="s">
-        <v>30</v>
+        <v>161</v>
       </c>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
       <c r="E24" s="20"/>
       <c r="F24" s="18"/>
-      <c r="G24" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
+      <c r="G24" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
     </row>
     <row r="25" spans="2:9" ht="15" customHeight="1">
       <c r="B25" s="19" t="s">
-        <v>31</v>
+        <v>162</v>
       </c>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
       <c r="E25" s="20"/>
       <c r="F25" s="18"/>
-      <c r="G25" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
+      <c r="G25" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
     </row>
     <row r="26" spans="2:9" ht="15" customHeight="1">
       <c r="B26" s="19" t="s">
-        <v>32</v>
+        <v>163</v>
       </c>
       <c r="C26" s="20"/>
       <c r="D26" s="20"/>
       <c r="E26" s="20"/>
       <c r="F26" s="18"/>
-      <c r="G26" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
+      <c r="G26" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
     </row>
     <row r="27" spans="2:9" ht="15" customHeight="1">
       <c r="B27" s="19" t="s">
-        <v>33</v>
+        <v>164</v>
       </c>
       <c r="C27" s="20"/>
       <c r="D27" s="20"/>
       <c r="E27" s="20"/>
       <c r="F27" s="18"/>
-      <c r="G27" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
+      <c r="G27" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
     </row>
     <row r="28" spans="2:9" ht="15" customHeight="1">
       <c r="B28" s="19" t="s">
-        <v>34</v>
+        <v>165</v>
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="20"/>
       <c r="E28" s="20"/>
       <c r="F28" s="18"/>
-      <c r="G28" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
+      <c r="G28" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
     </row>
     <row r="29" spans="2:9" ht="15" customHeight="1">
       <c r="B29" s="19" t="s">
-        <v>35</v>
+        <v>166</v>
       </c>
       <c r="C29" s="20"/>
       <c r="D29" s="20"/>
       <c r="E29" s="20"/>
       <c r="F29" s="18"/>
-      <c r="G29" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
+      <c r="G29" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
     </row>
     <row r="30" spans="2:9" ht="15" customHeight="1">
       <c r="B30" s="19" t="s">
-        <v>36</v>
+        <v>167</v>
       </c>
       <c r="C30" s="20"/>
       <c r="D30" s="20"/>
       <c r="E30" s="20"/>
       <c r="F30" s="18"/>
-      <c r="G30" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
+      <c r="G30" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
     </row>
     <row r="31" spans="2:9" ht="15" customHeight="1">
       <c r="B31" s="19" t="s">
-        <v>37</v>
+        <v>168</v>
       </c>
       <c r="C31" s="20"/>
       <c r="D31" s="20"/>
       <c r="E31" s="20"/>
       <c r="F31" s="18"/>
-      <c r="G31" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
+      <c r="G31" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
     </row>
     <row r="32" spans="2:9" ht="15" customHeight="1">
       <c r="B32" s="19" t="s">
-        <v>38</v>
+        <v>169</v>
       </c>
       <c r="C32" s="20"/>
       <c r="D32" s="20"/>
       <c r="E32" s="20"/>
       <c r="F32" s="18"/>
-      <c r="G32" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
+      <c r="G32" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
     </row>
     <row r="33" spans="2:9" ht="15" customHeight="1">
       <c r="B33" s="19" t="s">
-        <v>39</v>
+        <v>170</v>
       </c>
       <c r="C33" s="20"/>
       <c r="D33" s="20"/>
       <c r="E33" s="20"/>
       <c r="F33" s="18"/>
-      <c r="G33" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
+      <c r="G33" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
     </row>
     <row r="34" spans="2:9" ht="15" customHeight="1">
       <c r="B34" s="19" t="s">
-        <v>40</v>
+        <v>171</v>
       </c>
       <c r="C34" s="20"/>
       <c r="D34" s="20"/>
       <c r="E34" s="20"/>
       <c r="F34" s="18"/>
-      <c r="G34" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
+      <c r="G34" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
     </row>
     <row r="35" spans="2:9" ht="12.75" customHeight="1">
       <c r="B35" s="28" t="s">
-        <v>41</v>
+        <v>172</v>
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="20"/>
       <c r="E35" s="20"/>
       <c r="F35" s="18"/>
-      <c r="G35" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>15</v>
+      <c r="G35" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="36" spans="2:9" ht="15" customHeight="1">
       <c r="B36" s="19" t="s">
-        <v>42</v>
+        <v>173</v>
       </c>
       <c r="C36" s="20"/>
       <c r="D36" s="20"/>
       <c r="E36" s="20"/>
       <c r="F36" s="18"/>
-      <c r="G36" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
+      <c r="G36" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
     </row>
     <row r="37" spans="2:9" ht="15" customHeight="1">
       <c r="B37" s="19" t="s">
-        <v>43</v>
+        <v>174</v>
       </c>
       <c r="C37" s="20"/>
       <c r="D37" s="20"/>
       <c r="E37" s="20"/>
       <c r="F37" s="18"/>
-      <c r="G37" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
+      <c r="G37" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
     </row>
     <row r="38" spans="2:9" ht="15" customHeight="1">
       <c r="B38" s="19" t="s">
-        <v>44</v>
+        <v>175</v>
       </c>
       <c r="C38" s="20"/>
       <c r="D38" s="20"/>
       <c r="E38" s="20"/>
       <c r="F38" s="18"/>
-      <c r="G38" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
+      <c r="G38" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
     </row>
     <row r="39" spans="2:9" ht="15" customHeight="1">
       <c r="B39" s="19" t="s">
-        <v>45</v>
+        <v>176</v>
       </c>
       <c r="C39" s="20"/>
       <c r="D39" s="20"/>
       <c r="E39" s="20"/>
       <c r="F39" s="18"/>
-      <c r="G39" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
+      <c r="G39" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
     </row>
     <row r="40" spans="2:9" ht="27" customHeight="1">
       <c r="B40" s="24" t="s">
-        <v>46</v>
+        <v>177</v>
       </c>
       <c r="C40" s="20"/>
       <c r="D40" s="20"/>
@@ -4773,7 +4773,7 @@
     </row>
     <row r="41" spans="2:9" ht="66.75" customHeight="1">
       <c r="B41" s="25" t="s">
-        <v>47</v>
+        <v>178</v>
       </c>
       <c r="C41" s="20"/>
       <c r="D41" s="20"/>
@@ -4785,7 +4785,7 @@
     </row>
     <row r="42" spans="2:9" ht="30.75" customHeight="1">
       <c r="B42" s="24" t="s">
-        <v>48</v>
+        <v>179</v>
       </c>
       <c r="C42" s="20"/>
       <c r="D42" s="20"/>
@@ -4797,7 +4797,7 @@
     </row>
     <row r="43" spans="2:9" ht="77.25" customHeight="1">
       <c r="B43" s="25" t="s">
-        <v>49</v>
+        <v>180</v>
       </c>
       <c r="C43" s="20"/>
       <c r="D43" s="20"/>
@@ -4809,7 +4809,7 @@
     </row>
     <row r="44" spans="2:9" ht="27.75" customHeight="1">
       <c r="B44" s="24" t="s">
-        <v>50</v>
+        <v>181</v>
       </c>
       <c r="C44" s="20"/>
       <c r="D44" s="20"/>
@@ -4821,7 +4821,7 @@
     </row>
     <row r="45" spans="2:9" ht="63.75" customHeight="1">
       <c r="B45" s="25" t="s">
-        <v>47</v>
+        <v>178</v>
       </c>
       <c r="C45" s="20"/>
       <c r="D45" s="20"/>
@@ -4833,7 +4833,7 @@
     </row>
     <row r="46" spans="2:9" ht="28.5" customHeight="1">
       <c r="B46" s="24" t="s">
-        <v>51</v>
+        <v>182</v>
       </c>
       <c r="C46" s="20"/>
       <c r="D46" s="20"/>
@@ -4845,7 +4845,7 @@
     </row>
     <row r="47" spans="2:9" ht="64.5" customHeight="1">
       <c r="B47" s="21" t="s">
-        <v>52</v>
+        <v>183</v>
       </c>
       <c r="C47" s="22"/>
       <c r="D47" s="22"/>
@@ -4856,30 +4856,30 @@
       <c r="I47" s="23"/>
     </row>
     <row r="48" spans="2:9" ht="33" customHeight="1">
-      <c r="B48" s="6"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="12" t="s">
-        <v>53</v>
+      <c r="B48" s="5"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="11" t="s">
+        <v>184</v>
       </c>
       <c r="G48" s="32" t="s">
-        <v>54</v>
+        <v>185</v>
       </c>
       <c r="H48" s="20"/>
       <c r="I48" s="18"/>
     </row>
     <row r="49" spans="2:9" ht="36" customHeight="1">
-      <c r="B49" s="8"/>
-      <c r="C49" s="9"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="8"/>
       <c r="D49" s="26" t="s">
-        <v>55</v>
+        <v>186</v>
       </c>
       <c r="E49" s="20"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="9"/>
-      <c r="H49" s="9"/>
-      <c r="I49" s="10"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="I49" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="48">
@@ -4934,7 +4934,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="74" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="77" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>